<commit_message>
Update Finviz breadth data
</commit_message>
<xml_diff>
--- a/finviz_breadth.xlsx
+++ b/finviz_breadth.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -995,6 +995,53 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>101</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>44.1%</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>128</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>55.9%</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2824</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>50.2%</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2534</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>45.0%</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>